<commit_message>
Result filter & swagger added in backend & Folder allocation changes
</commit_message>
<xml_diff>
--- a/Studies.xlsx
+++ b/Studies.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PK\Project\Shopping-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193E2EF1-1428-4BB3-AE74-687F7BD7234D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ECE5D0B-6FEE-4AB4-8FA8-D0EC8DB11EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="130">
   <si>
     <t>Backend Topics</t>
   </si>
@@ -171,12 +171,6 @@
     <t>safe navigation -&gt; User?.name</t>
   </si>
   <si>
-    <t>sealed , singleton</t>
-  </si>
-  <si>
-    <t>abstract</t>
-  </si>
-  <si>
     <t>final , finally , finalize</t>
   </si>
   <si>
@@ -279,13 +273,7 @@
     <t>Signals , Computed , writable</t>
   </si>
   <si>
-    <t>Testing</t>
-  </si>
-  <si>
     <t>React</t>
-  </si>
-  <si>
-    <t>How to get the values from excel sheet</t>
   </si>
   <si>
     <t>PPT</t>
@@ -394,9 +382,6 @@
     <t>JWT decode</t>
   </si>
   <si>
-    <t xml:space="preserve">Ng for , ng if </t>
-  </si>
-  <si>
     <t>SOLID</t>
   </si>
   <si>
@@ -440,6 +425,9 @@
   </si>
   <si>
     <t>Debounce</t>
+  </si>
+  <si>
+    <t>sealed , singleton ,abstract</t>
   </si>
 </sst>
 </file>
@@ -553,7 +541,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -857,7 +845,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -866,16 +854,16 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="10" t="s">
         <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
@@ -883,26 +871,26 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="10" t="s">
         <v>20</v>
       </c>
     </row>
@@ -913,7 +901,7 @@
       <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="10" t="s">
         <v>21</v>
       </c>
     </row>
@@ -924,7 +912,7 @@
       <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="10" t="s">
         <v>39</v>
       </c>
     </row>
@@ -936,7 +924,7 @@
         <v>28</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -946,7 +934,7 @@
       <c r="B8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="10" t="s">
         <v>40</v>
       </c>
     </row>
@@ -957,7 +945,7 @@
       <c r="B9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="10" t="s">
         <v>41</v>
       </c>
     </row>
@@ -968,29 +956,29 @@
       <c r="B10" t="s">
         <v>31</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="10" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="10" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B12" t="s">
         <v>33</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="10" t="s">
         <v>44</v>
       </c>
     </row>
@@ -999,10 +987,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1010,10 +998,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1021,10 +1009,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1032,10 +1020,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1043,18 +1031,18 @@
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C18" t="s">
-        <v>56</v>
+      <c r="C18" s="10" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -1062,10 +1050,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1073,59 +1061,59 @@
         <v>17</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="C20" t="s">
-        <v>58</v>
+        <v>114</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="10" t="s">
         <v>34</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" t="s">
-        <v>59</v>
+        <v>114</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="10" t="s">
         <v>35</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="C22" t="s">
-        <v>68</v>
+        <v>114</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
-      <c r="C23" t="s">
-        <v>69</v>
+      <c r="C23" s="10" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
-      <c r="C24" t="s">
-        <v>70</v>
+      <c r="C24" s="10" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="10" t="s">
         <v>38</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="C25" t="s">
-        <v>71</v>
+        <v>119</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -1133,10 +1121,10 @@
         <v>45</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C26" t="s">
-        <v>72</v>
+        <v>120</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -1144,232 +1132,223 @@
         <v>46</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="3" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C31" s="3" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>49</v>
-      </c>
-      <c r="C30" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>50</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>79</v>
+        <v>59</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>65</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>84</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="C37" s="4"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>86</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="C38" s="4"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>96</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>100</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>106</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>107</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>108</v>
+        <v>103</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>120</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>110</v>
+        <v>115</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>121</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>111</v>
+        <v>116</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>122</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>112</v>
+        <v>117</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>128</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>115</v>
+        <v>123</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C53" s="4" t="s">
-        <v>116</v>
+      <c r="C53" s="10" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C54" s="4" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C55" s="4" t="s">
-        <v>118</v>
-      </c>
+      <c r="C55" s="4"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C56" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C57" s="10" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>